<commit_message>
Actualiza el calendario con la columna Link
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015vEhi5mBHxnpU6v1gxnGGU
</commit_message>
<xml_diff>
--- a/datos/calendario.xlsx
+++ b/datos/calendario.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elena.ojeda\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oscar.nieto/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A2043A02-6178-4452-A046-1E800CC4AD39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CBA9C74-44F6-C148-96F0-62930883C1B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31140" yWindow="0" windowWidth="24675" windowHeight="15585" xr2:uid="{19026AE3-6B4F-45D3-8604-4731C2D808B9}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{19026AE3-6B4F-45D3-8604-4731C2D808B9}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="40">
   <si>
     <t>Fecha</t>
   </si>
@@ -153,6 +153,12 @@
   </si>
   <si>
     <t>29, 30 ,1 y 2 /09 y 10/2026</t>
+  </si>
+  <si>
+    <t>https://www.google.com/</t>
+  </si>
+  <si>
+    <t>Link</t>
   </si>
 </sst>
 </file>
@@ -220,18 +226,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -240,7 +241,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -578,22 +579,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED011342-C7D1-41BA-9CA2-E06902A80352}">
-  <dimension ref="A3:F13"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A3:G13"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="51.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="51.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.1640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="49.36328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="49.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="5" t="s">
         <v>0</v>
       </c>
       <c r="C3" s="1" t="s">
@@ -608,93 +610,98 @@
       <c r="F3" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
+      <c r="G3" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2" t="s">
+      <c r="E4" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
+      <c r="G4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="6">
+      <c r="B5" s="4">
         <v>46280</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="9">
+      <c r="D5" s="6">
         <v>0.79166666666666663</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" t="s">
         <v>20</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F5" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="6">
+      <c r="B6" s="4">
         <v>46281</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="9">
+      <c r="D6" s="6">
         <v>0.79166666666666663</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" t="s">
         <v>19</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="7">
+      <c r="B7" s="4">
         <v>46282</v>
       </c>
       <c r="C7" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="2">
         <v>0.79166666666666663</v>
       </c>
       <c r="E7" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>24</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="4" t="s">
         <v>25</v>
       </c>
       <c r="C8" t="s">
         <v>26</v>
       </c>
-      <c r="D8" s="4"/>
+      <c r="D8" s="2"/>
       <c r="E8" t="s">
         <v>12</v>
       </c>
@@ -702,64 +709,64 @@
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="7">
+      <c r="B9" s="4">
         <v>46289</v>
       </c>
       <c r="C9" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="2" t="s">
         <v>23</v>
       </c>
       <c r="E9" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>28</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="4" t="s">
         <v>37</v>
       </c>
       <c r="C10" t="s">
         <v>29</v>
       </c>
-      <c r="D10" s="4"/>
+      <c r="D10" s="2"/>
       <c r="E10" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="7">
+      <c r="B11" s="4">
         <v>46294</v>
       </c>
       <c r="C11" t="s">
         <v>36</v>
       </c>
-      <c r="D11" s="4"/>
+      <c r="D11" s="2"/>
       <c r="E11" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="7">
+      <c r="B12" s="4">
         <v>46295</v>
       </c>
       <c r="C12" t="s">
         <v>35</v>
       </c>
-      <c r="D12" s="4"/>
+      <c r="D12" s="2"/>
       <c r="E12" t="s">
         <v>12</v>
       </c>
@@ -767,17 +774,17 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>31</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="4" t="s">
         <v>32</v>
       </c>
       <c r="C13" t="s">
         <v>29</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E13" t="s">

</xml_diff>